<commit_message>
Ingles: documenta prova oral na skill e adiciona observacao no calendario
Skill (calendario-provas/SKILL.md): novo item 16 no Passo 0 -- a prova
de Ingles do calendario normal e so a escrita; a prova oral precisa
de dia(s) a parte, decididos pela propria equipe de Ingles (nunca
inferir ou sugerir essas datas). Toda entrega de calendario deve
incluir uma observacao visivel na planilha sobre isso.

Proposta 3: adicionada observacao nas 8 turmas, na area de "DATAS
IMPORTANTES" ja existente (colunas L/M), com destaque de cor: "Ingles
-- Prova oral: precisa de dia(s) a parte da prova escrita ja no
calendario; a equipe de Ingles deve sinalizar as datas de aplicacao".

verificar_calendario.py: 6 PROBLEMA ja conhecidos e autorizados,
nenhum novo -- mudanca nao mexeu na grade de provas, so adicionou
celula informativa fora da area de alocacao.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -264,7 +264,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill/>
     </fill>
@@ -455,6 +455,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE7E6E6"/>
         <bgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
+        <bgColor rgb="FFDCE6F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -1848,7 +1854,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="472">
+  <cellXfs count="473">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -3456,6 +3462,9 @@
     <xf numFmtId="0" fontId="5" fillId="27" borderId="25" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -6113,7 +6122,7 @@
           <t>unterrichtsfrei sem aula</t>
         </is>
       </c>
-      <c r="F18" s="468" t="inlineStr">
+      <c r="F18" s="470" t="inlineStr">
         <is>
           <t>Hist - Wag
 10º e 11º tempos</t>
@@ -6138,7 +6147,7 @@
       <c r="C19" s="313" t="n"/>
       <c r="D19" s="314" t="n"/>
       <c r="E19" s="315" t="n"/>
-      <c r="F19" s="406" t="n"/>
+      <c r="F19" s="437" t="n"/>
       <c r="I19" s="383" t="n"/>
       <c r="J19" s="315" t="n"/>
       <c r="L19" s="29" t="inlineStr">
@@ -6159,7 +6168,7 @@
       <c r="C20" s="313" t="n"/>
       <c r="D20" s="314" t="n"/>
       <c r="E20" s="315" t="n"/>
-      <c r="F20" s="407" t="n"/>
+      <c r="F20" s="439" t="n"/>
       <c r="I20" s="384" t="n"/>
       <c r="J20" s="315" t="n"/>
       <c r="L20" s="29" t="n"/>
@@ -6661,6 +6670,16 @@
       <c r="H38" s="439" t="n"/>
       <c r="I38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
+      <c r="L38" s="472" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="M38" s="472" t="inlineStr">
+        <is>
+          <t>Inglês — Prova oral: precisa de dia(s) à parte da prova escrita já no calendário; a equipe de Inglês deve sinalizar as datas de aplicação</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A39" s="119">
@@ -9859,6 +9878,16 @@
       <c r="H38" s="439" t="n"/>
       <c r="I38" s="438" t="n"/>
       <c r="J38" s="352" t="n"/>
+      <c r="L38" s="472" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="M38" s="472" t="inlineStr">
+        <is>
+          <t>Inglês — Prova oral: precisa de dia(s) à parte da prova escrita já no calendário; a equipe de Inglês deve sinalizar as datas de aplicação</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A39" s="119">
@@ -11537,6 +11566,16 @@
       <c r="H38" s="439" t="n"/>
       <c r="I38" s="438" t="n"/>
       <c r="J38" s="352" t="n"/>
+      <c r="L38" s="472" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="M38" s="472" t="inlineStr">
+        <is>
+          <t>Inglês — Prova oral: precisa de dia(s) à parte da prova escrita já no calendário; a equipe de Inglês deve sinalizar as datas de aplicação</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A39" s="119">
@@ -13221,6 +13260,16 @@
       <c r="G38" s="439" t="n"/>
       <c r="H38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
+      <c r="L38" s="472" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="M38" s="472" t="inlineStr">
+        <is>
+          <t>Inglês — Prova oral: precisa de dia(s) à parte da prova escrita já no calendário; a equipe de Inglês deve sinalizar as datas de aplicação</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A39" s="119">
@@ -14900,6 +14949,16 @@
       <c r="H38" s="439" t="n"/>
       <c r="I38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
+      <c r="L38" s="472" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="M38" s="472" t="inlineStr">
+        <is>
+          <t>Inglês — Prova oral: precisa de dia(s) à parte da prova escrita já no calendário; a equipe de Inglês deve sinalizar as datas de aplicação</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A39" s="119">
@@ -16592,6 +16651,16 @@
       <c r="H38" s="283" t="n"/>
       <c r="I38" s="438" t="n"/>
       <c r="J38" s="352" t="n"/>
+      <c r="L38" s="472" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="M38" s="472" t="inlineStr">
+        <is>
+          <t>Inglês — Prova oral: precisa de dia(s) à parte da prova escrita já no calendário; a equipe de Inglês deve sinalizar as datas de aplicação</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A39" s="119">
@@ -18292,6 +18361,16 @@
       <c r="H38" s="283" t="n"/>
       <c r="I38" s="438" t="n"/>
       <c r="J38" s="352" t="n"/>
+      <c r="L38" s="472" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="M38" s="472" t="inlineStr">
+        <is>
+          <t>Inglês — Prova oral: precisa de dia(s) à parte da prova escrita já no calendário; a equipe de Inglês deve sinalizar as datas de aplicação</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A39" s="119">
@@ -20024,6 +20103,16 @@
       <c r="H38" s="439" t="n"/>
       <c r="I38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
+      <c r="L38" s="472" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="M38" s="472" t="inlineStr">
+        <is>
+          <t>Inglês — Prova oral: precisa de dia(s) à parte da prova escrita já no calendário; a equipe de Inglês deve sinalizar as datas de aplicação</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A39" s="119">

</xml_diff>

<commit_message>
10C: Geografia (1a prova) para tempos 2-3, mesmo dia (11/09)
Geografia (10C1+10C2): semana6 sexta (11/09), bloco 1o-2o -> 2o-3o
tempos. GL deixa de doar (estava no teto de 3 cessoes nas duas
turmas); Alemao/DaF passa a doar (6->7 cessoes, exatamente no teto
por percentual, sem estourar).

verificar_calendario.py fecha so com os 6 PROBLEMA ja conhecidos e
autorizados -- nenhum novo. 1 AVISO leve novo por turma (DaF cede na
propria semana da prova dela). Distancia entre as 2 ocorrencias de
Geografia inalterada. 5 relatorios regenerados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -12728,10 +12728,10 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="I18" s="423" t="inlineStr">
+      <c r="I18" s="442" t="inlineStr">
         <is>
           <t>Geo - Mlo
-1º e 2º tempos</t>
+2º e 3º tempos</t>
         </is>
       </c>
       <c r="J18" s="183" t="n"/>
@@ -12748,7 +12748,7 @@
       <c r="F19" s="222" t="n"/>
       <c r="G19" s="437" t="n"/>
       <c r="H19" s="437" t="n"/>
-      <c r="I19" s="383" t="n"/>
+      <c r="I19" s="437" t="n"/>
       <c r="J19" s="315" t="n"/>
       <c r="L19" s="29" t="inlineStr">
         <is>
@@ -12771,7 +12771,7 @@
       <c r="F20" s="222" t="n"/>
       <c r="G20" s="439" t="n"/>
       <c r="H20" s="439" t="n"/>
-      <c r="I20" s="384" t="n"/>
+      <c r="I20" s="439" t="n"/>
       <c r="J20" s="315" t="n"/>
       <c r="L20" s="29" t="n"/>
       <c r="M20" s="29" t="n"/>
@@ -14419,10 +14419,10 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="I18" s="423" t="inlineStr">
+      <c r="I18" s="410" t="inlineStr">
         <is>
           <t>Geo - Mlo
-1º e 2º tempos</t>
+2º e 3º tempos</t>
         </is>
       </c>
       <c r="J18" s="183" t="n"/>
@@ -14439,7 +14439,7 @@
       <c r="F19" s="222" t="n"/>
       <c r="G19" s="437" t="n"/>
       <c r="H19" s="437" t="n"/>
-      <c r="I19" s="383" t="n"/>
+      <c r="I19" s="406" t="n"/>
       <c r="J19" s="315" t="n"/>
       <c r="L19" s="29" t="inlineStr">
         <is>
@@ -14462,7 +14462,7 @@
       <c r="F20" s="222" t="n"/>
       <c r="G20" s="439" t="n"/>
       <c r="H20" s="439" t="n"/>
-      <c r="I20" s="384" t="n"/>
+      <c r="I20" s="407" t="n"/>
       <c r="J20" s="315" t="n"/>
       <c r="L20" s="29" t="n"/>
       <c r="M20" s="29" t="n"/>

</xml_diff>

<commit_message>
12C1/12C2: reposiciona DaF e GL (2a prova) para semana 14
DaF: 23/10 -> 06/11 (sexta, 6o-7o tempos, mesmo bloco de aula dupla real).
GL: 01/10 -> 05/11 (quinta, 9o-10o tempos, mesmo bloco).

06/10 foi descartado por analise: DaF nao tem aula com 12C1/12C2 as
tercas-feiras, so segunda (4o tempo) e sexta (6o-7o tempos). Portugues
(LP/LIT/RED) permanece em 09/10, sem alteracao.

Testado em copia isolada antes de aplicar: verificar_calendario.py sem
nenhum PROBLEMA novo, so 2 AVISOs leves esperados (DaF cede tempo na
mesma semana da propria prova - e a cessao que libera a semana para as
duas provas). Distancia entre as duas ocorrencias de DaF sobe de 5 para
7 semanas; a de GL sobe de 4 para 9 semanas.

Os 5 relatorios derivados foram regenerados e o historico documentado
em referencia/estado_2sem_2026.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018hTHGw5BjMp2kfES5oHVby
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6362,12 +6362,7 @@
       <c r="E27" s="464" t="n"/>
       <c r="F27" s="283" t="n"/>
       <c r="G27" s="435" t="n"/>
-      <c r="H27" s="436" t="inlineStr">
-        <is>
-          <t>GL - CBu-EFr-Eth
-9º e 10º tempos</t>
-        </is>
-      </c>
+      <c r="H27" s="183" t="n"/>
       <c r="I27" s="435" t="n"/>
       <c r="J27" s="265" t="n"/>
       <c r="L27" s="45" t="n"/>
@@ -6386,7 +6381,7 @@
       <c r="E28" s="438" t="n"/>
       <c r="F28" s="283" t="n"/>
       <c r="G28" s="438" t="n"/>
-      <c r="H28" s="437" t="n"/>
+      <c r="H28" s="315" t="n"/>
       <c r="I28" s="438" t="n"/>
       <c r="J28" s="352" t="n"/>
       <c r="L28" s="23" t="n"/>
@@ -6405,7 +6400,7 @@
       <c r="E29" s="438" t="n"/>
       <c r="F29" s="283" t="n"/>
       <c r="G29" s="438" t="n"/>
-      <c r="H29" s="439" t="n"/>
+      <c r="H29" s="315" t="n"/>
       <c r="I29" s="438" t="n"/>
       <c r="J29" s="352" t="n"/>
       <c r="L29" s="46" t="n"/>
@@ -6621,12 +6616,7 @@
 5º e 6º tempos</t>
         </is>
       </c>
-      <c r="I36" s="443" t="inlineStr">
-        <is>
-          <t>DaF - CBu-EFr-Eth
-6º e 7º tempos</t>
-        </is>
-      </c>
+      <c r="I36" s="183" t="n"/>
       <c r="J36" s="265" t="n"/>
       <c r="L36" s="81" t="inlineStr">
         <is>
@@ -6647,7 +6637,7 @@
       <c r="E37" s="283" t="n"/>
       <c r="F37" s="437" t="n"/>
       <c r="H37" s="437" t="n"/>
-      <c r="I37" s="437" t="n"/>
+      <c r="I37" s="315" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
@@ -6668,7 +6658,7 @@
       <c r="E38" s="283" t="n"/>
       <c r="F38" s="439" t="n"/>
       <c r="H38" s="439" t="n"/>
-      <c r="I38" s="439" t="n"/>
+      <c r="I38" s="315" t="n"/>
       <c r="J38" s="352" t="n"/>
       <c r="L38" s="472" t="inlineStr">
         <is>
@@ -6769,8 +6759,18 @@
 4º tempo</t>
         </is>
       </c>
-      <c r="H42" s="283" t="n"/>
-      <c r="I42" s="451" t="n"/>
+      <c r="H42" s="436" t="inlineStr">
+        <is>
+          <t>GL - CBu-EFr-Eth
+9º e 10º tempos</t>
+        </is>
+      </c>
+      <c r="I42" s="443" t="inlineStr">
+        <is>
+          <t>DaF - CBu-EFr-Eth
+6º e 7º tempos</t>
+        </is>
+      </c>
       <c r="J42" s="265" t="n"/>
       <c r="L42" s="259" t="inlineStr">
         <is>
@@ -6786,7 +6786,8 @@
       <c r="D43" s="350" t="n"/>
       <c r="E43" s="283" t="n"/>
       <c r="G43" s="437" t="n"/>
-      <c r="H43" s="283" t="n"/>
+      <c r="H43" s="437" t="n"/>
+      <c r="I43" s="437" t="n"/>
       <c r="J43" s="352" t="n"/>
       <c r="L43" s="331" t="n"/>
     </row>
@@ -6797,7 +6798,8 @@
       <c r="D44" s="350" t="n"/>
       <c r="E44" s="283" t="n"/>
       <c r="G44" s="439" t="n"/>
-      <c r="H44" s="283" t="n"/>
+      <c r="H44" s="439" t="n"/>
+      <c r="I44" s="439" t="n"/>
       <c r="J44" s="352" t="n"/>
       <c r="L44" s="331" t="n"/>
     </row>
@@ -7119,7 +7121,7 @@
       <c r="J62" s="353" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="169">
+  <mergeCells count="171">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="G54:G56"/>
     <mergeCell ref="C21:C23"/>
@@ -7177,6 +7179,7 @@
     <mergeCell ref="E12:E14"/>
     <mergeCell ref="J33:J35"/>
     <mergeCell ref="E21:E23"/>
+    <mergeCell ref="H42:H44"/>
     <mergeCell ref="J42:J44"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="J60:J62"/>
@@ -7204,6 +7207,7 @@
     <mergeCell ref="A18:A20"/>
     <mergeCell ref="E9:E11"/>
     <mergeCell ref="C27:C29"/>
+    <mergeCell ref="I42:I44"/>
     <mergeCell ref="B15:B17"/>
     <mergeCell ref="B24:B26"/>
     <mergeCell ref="D24:D26"/>
@@ -14419,7 +14423,7 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="I18" s="410" t="inlineStr">
+      <c r="I18" s="442" t="inlineStr">
         <is>
           <t>Geo - Mlo
 2º e 3º tempos</t>
@@ -14439,7 +14443,7 @@
       <c r="F19" s="222" t="n"/>
       <c r="G19" s="437" t="n"/>
       <c r="H19" s="437" t="n"/>
-      <c r="I19" s="406" t="n"/>
+      <c r="I19" s="437" t="n"/>
       <c r="J19" s="315" t="n"/>
       <c r="L19" s="29" t="inlineStr">
         <is>
@@ -14462,7 +14466,7 @@
       <c r="F20" s="222" t="n"/>
       <c r="G20" s="439" t="n"/>
       <c r="H20" s="439" t="n"/>
-      <c r="I20" s="407" t="n"/>
+      <c r="I20" s="439" t="n"/>
       <c r="J20" s="315" t="n"/>
       <c r="L20" s="29" t="n"/>
       <c r="M20" s="29" t="n"/>
@@ -19795,12 +19799,7 @@
       <c r="E27" s="78" t="n"/>
       <c r="F27" s="283" t="n"/>
       <c r="G27" s="435" t="n"/>
-      <c r="H27" s="436" t="inlineStr">
-        <is>
-          <t>GL - CBu-EFr-Eth
-9º e 10º tempos</t>
-        </is>
-      </c>
+      <c r="H27" s="183" t="n"/>
       <c r="I27" s="435" t="n"/>
       <c r="J27" s="265" t="n"/>
       <c r="L27" s="45" t="n"/>
@@ -19819,7 +19818,7 @@
       <c r="E28" s="78" t="n"/>
       <c r="F28" s="283" t="n"/>
       <c r="G28" s="438" t="n"/>
-      <c r="H28" s="437" t="n"/>
+      <c r="H28" s="315" t="n"/>
       <c r="I28" s="438" t="n"/>
       <c r="J28" s="352" t="n"/>
       <c r="L28" s="23" t="n"/>
@@ -19838,7 +19837,7 @@
       <c r="E29" s="78" t="n"/>
       <c r="F29" s="283" t="n"/>
       <c r="G29" s="438" t="n"/>
-      <c r="H29" s="439" t="n"/>
+      <c r="H29" s="315" t="n"/>
       <c r="I29" s="438" t="n"/>
       <c r="J29" s="352" t="n"/>
       <c r="L29" s="46" t="n"/>
@@ -20054,12 +20053,7 @@
 5º e 6º tempos</t>
         </is>
       </c>
-      <c r="I36" s="443" t="inlineStr">
-        <is>
-          <t>DaF - CBu-EFr-Eth
-6º e 7º tempos</t>
-        </is>
-      </c>
+      <c r="I36" s="183" t="n"/>
       <c r="J36" s="265" t="n"/>
       <c r="L36" s="81" t="inlineStr">
         <is>
@@ -20080,7 +20074,7 @@
       <c r="E37" s="283" t="n"/>
       <c r="F37" s="437" t="n"/>
       <c r="H37" s="437" t="n"/>
-      <c r="I37" s="437" t="n"/>
+      <c r="I37" s="315" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
@@ -20101,7 +20095,7 @@
       <c r="E38" s="283" t="n"/>
       <c r="F38" s="439" t="n"/>
       <c r="H38" s="439" t="n"/>
-      <c r="I38" s="439" t="n"/>
+      <c r="I38" s="315" t="n"/>
       <c r="J38" s="352" t="n"/>
       <c r="L38" s="472" t="inlineStr">
         <is>
@@ -20202,8 +20196,18 @@
 10º tempo</t>
         </is>
       </c>
-      <c r="H42" s="435" t="n"/>
-      <c r="I42" s="451" t="n"/>
+      <c r="H42" s="436" t="inlineStr">
+        <is>
+          <t>GL - CBu-EFr-Eth
+9º e 10º tempos</t>
+        </is>
+      </c>
+      <c r="I42" s="443" t="inlineStr">
+        <is>
+          <t>DaF - CBu-EFr-Eth
+6º e 7º tempos</t>
+        </is>
+      </c>
       <c r="J42" s="265" t="n"/>
       <c r="L42" s="259" t="inlineStr">
         <is>
@@ -20219,7 +20223,8 @@
       <c r="D43" s="350" t="n"/>
       <c r="E43" s="283" t="n"/>
       <c r="G43" s="437" t="n"/>
-      <c r="H43" s="438" t="n"/>
+      <c r="H43" s="437" t="n"/>
+      <c r="I43" s="437" t="n"/>
       <c r="J43" s="352" t="n"/>
       <c r="L43" s="331" t="n"/>
     </row>
@@ -20230,7 +20235,8 @@
       <c r="D44" s="350" t="n"/>
       <c r="E44" s="283" t="n"/>
       <c r="G44" s="439" t="n"/>
-      <c r="H44" s="438" t="n"/>
+      <c r="H44" s="439" t="n"/>
+      <c r="I44" s="439" t="n"/>
       <c r="J44" s="352" t="n"/>
       <c r="L44" s="331" t="n"/>
     </row>
@@ -20552,7 +20558,7 @@
       <c r="J62" s="353" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="169">
+  <mergeCells count="171">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="G54:G56"/>
     <mergeCell ref="C21:C23"/>
@@ -20610,6 +20616,7 @@
     <mergeCell ref="E12:E14"/>
     <mergeCell ref="J33:J35"/>
     <mergeCell ref="E21:E23"/>
+    <mergeCell ref="H42:H44"/>
     <mergeCell ref="J42:J44"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="J60:J62"/>
@@ -20637,6 +20644,7 @@
     <mergeCell ref="A18:A20"/>
     <mergeCell ref="E9:E11"/>
     <mergeCell ref="C27:C29"/>
+    <mergeCell ref="I42:I44"/>
     <mergeCell ref="B15:B17"/>
     <mergeCell ref="B24:B26"/>
     <mergeCell ref="D24:D26"/>

</xml_diff>

<commit_message>
9C1/9C2: move Matematica (2a prova) de 19/11 para 24/11
Segunda nao tem aula de Mat em nenhuma das duas turmas (inviavel por
prioridade 1); quarta exigiria ceder o bloco duplo inteiro de
Gramatica na 9C2. Terca (9o-10o tempos) e tempo proprio do prof. BrSa
em pelo menos uma das turmas em cada posicao do bloco (9C1 no 9o, 9C2
no 10o) - cessao minima dos dois lados.

Resultado: nenhum PROBLEMA novo, e 2 AVISOs a menos (Artes voltou a
ceder dentro do teto de 2, sem precisar doar tempo para o bloco antigo
de quinta). A semana 17 (9C1/9C2), que ficava vazia de proposito,
passa a ter prova antes de quarta, cumprindo essa regra por si so.
Distancia da 1a prova de Matematica sobe de 9 para 10 semanas.

Testado em copia isolada antes de aplicar. Os 5 relatorios derivados
foram regenerados e o historico documentado em
referencia/estado_2sem_2026.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018hTHGw5BjMp2kfES5oHVby
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -10108,12 +10108,7 @@
         </is>
       </c>
       <c r="G48" s="441" t="n"/>
-      <c r="H48" s="441" t="inlineStr">
-        <is>
-          <t>Mat - BrSa
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="H48" s="183" t="n"/>
       <c r="I48" s="183" t="inlineStr">
         <is>
           <t>unterrichtsfrei sem aula</t>
@@ -10127,7 +10122,7 @@
       <c r="C49" s="313" t="n"/>
       <c r="D49" s="350" t="n"/>
       <c r="F49" s="437" t="n"/>
-      <c r="H49" s="437" t="n"/>
+      <c r="H49" s="315" t="n"/>
       <c r="I49" s="315" t="n"/>
       <c r="J49" s="352" t="n"/>
     </row>
@@ -10137,7 +10132,7 @@
       <c r="C50" s="313" t="n"/>
       <c r="D50" s="350" t="n"/>
       <c r="F50" s="439" t="n"/>
-      <c r="H50" s="439" t="n"/>
+      <c r="H50" s="315" t="n"/>
       <c r="I50" s="315" t="n"/>
       <c r="J50" s="352" t="n"/>
     </row>
@@ -10160,7 +10155,12 @@
         <v/>
       </c>
       <c r="E51" s="435" t="n"/>
-      <c r="F51" s="183" t="n"/>
+      <c r="F51" s="441" t="inlineStr">
+        <is>
+          <t>Mat - BrSa
+9º e 10º tempos</t>
+        </is>
+      </c>
       <c r="G51" s="183" t="n"/>
       <c r="H51" s="183" t="n"/>
       <c r="I51" s="386" t="inlineStr">
@@ -10177,7 +10177,7 @@
       <c r="C52" s="313" t="n"/>
       <c r="D52" s="350" t="n"/>
       <c r="E52" s="438" t="n"/>
-      <c r="F52" s="315" t="n"/>
+      <c r="F52" s="437" t="n"/>
       <c r="G52" s="315" t="n"/>
       <c r="H52" s="315" t="n"/>
       <c r="I52" s="351" t="n"/>
@@ -10189,7 +10189,7 @@
       <c r="C53" s="313" t="n"/>
       <c r="D53" s="350" t="n"/>
       <c r="E53" s="438" t="n"/>
-      <c r="F53" s="315" t="n"/>
+      <c r="F53" s="439" t="n"/>
       <c r="G53" s="315" t="n"/>
       <c r="H53" s="315" t="n"/>
       <c r="I53" s="387" t="n"/>
@@ -11796,12 +11796,7 @@
         </is>
       </c>
       <c r="G48" s="441" t="n"/>
-      <c r="H48" s="441" t="inlineStr">
-        <is>
-          <t>Mat - BrSa
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="H48" s="183" t="n"/>
       <c r="I48" s="183" t="inlineStr">
         <is>
           <t>unterrichtsfrei sem aula</t>
@@ -11815,7 +11810,7 @@
       <c r="C49" s="313" t="n"/>
       <c r="D49" s="350" t="n"/>
       <c r="F49" s="437" t="n"/>
-      <c r="H49" s="437" t="n"/>
+      <c r="H49" s="315" t="n"/>
       <c r="I49" s="315" t="n"/>
       <c r="J49" s="352" t="n"/>
     </row>
@@ -11825,7 +11820,7 @@
       <c r="C50" s="313" t="n"/>
       <c r="D50" s="350" t="n"/>
       <c r="F50" s="439" t="n"/>
-      <c r="H50" s="439" t="n"/>
+      <c r="H50" s="315" t="n"/>
       <c r="I50" s="315" t="n"/>
       <c r="J50" s="352" t="n"/>
     </row>
@@ -11848,7 +11843,12 @@
         <v/>
       </c>
       <c r="E51" s="435" t="n"/>
-      <c r="F51" s="183" t="n"/>
+      <c r="F51" s="441" t="inlineStr">
+        <is>
+          <t>Mat - BrSa
+9º e 10º tempos</t>
+        </is>
+      </c>
       <c r="G51" s="183" t="n"/>
       <c r="H51" s="183" t="n"/>
       <c r="I51" s="386" t="inlineStr">
@@ -11865,7 +11865,7 @@
       <c r="C52" s="313" t="n"/>
       <c r="D52" s="350" t="n"/>
       <c r="E52" s="438" t="n"/>
-      <c r="F52" s="315" t="n"/>
+      <c r="F52" s="437" t="n"/>
       <c r="G52" s="315" t="n"/>
       <c r="H52" s="315" t="n"/>
       <c r="I52" s="351" t="n"/>
@@ -11877,7 +11877,7 @@
       <c r="C53" s="313" t="n"/>
       <c r="D53" s="350" t="n"/>
       <c r="E53" s="438" t="n"/>
-      <c r="F53" s="315" t="n"/>
+      <c r="F53" s="439" t="n"/>
       <c r="G53" s="315" t="n"/>
       <c r="H53" s="315" t="n"/>
       <c r="I53" s="387" t="n"/>

</xml_diff>